<commit_message>
Add 45-second Evan Lange script versions to TikTok scripts spreadsheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012RwHDQ9KSjMEpyGbxMwsiX
</commit_message>
<xml_diff>
--- a/tiktok_scripts.xlsx
+++ b/tiktok_scripts.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scripts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Evan Lange 45s" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scripts" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,6 +427,500 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:G15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="100" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Tema</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Hook (sin cambios)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Script completo (para grabar)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Palabras</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Duración est. (s)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Video original</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>PIP</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>When an employee receives a PIP, also known as a performance improvement plan, in most cases, they will be fired.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>When an employee receives a PIP, also known as a performance improvement plan, in most cases, they will be fired. I'm Evan Lange, with one of Texas's top-rated employment law firms. A PIP lists the areas where you're supposedly falling short and gives you a deadline, often 30, 60 or 90 days, to fix them. The problem? Many times the decision has already been made, and the PIP becomes the company's proof that they warned you. So if you get one, take it seriously. Keep copies of everything, respond in writing to anything inaccurate, and if it showed up right after you complained or asked for leave, talk to an employment lawyer before your deadline runs out.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>117</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@craigleveyesq/video/7693280124254440735</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Second job</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Can you get fired by your company because you have more than one job? In many cases the answer is yes.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Can you get fired by your company because you have more than one job? In many cases the answer is yes. I'm Evan Lange, with one of Texas's top-rated employment law firms. Texas is an at-will state, so your employer can let you go for almost any reason that isn't illegal, and having a second job isn't a protected reason. Check your handbook for a moonlighting or outside-employment policy, and read your offer letter for conflict-of-interest or non-compete language. The biggest risks: working for a competitor, using company time or equipment, or letting your performance slip. Not sure? Get approval in writing before you start.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>105</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@craigleveyesq/video/7692562235637435679</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Before you resign</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>If I was an employee that was about to resign from their job, here are three things that I would not do.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>If I was an employee that was about to resign from their job, here are three things that I would not do. I'm Evan Lange, with one of Texas's top-rated employment law firms. One: don't give notice until your new offer is signed and your background check has cleared. If the new job falls through, you could end up with nothing. Two: don't pick your last day at random. Check when bonuses, commissions and vesting dates hit so you don't leave earned money behind. Three: don't count on working out your two weeks. Many employers can end things the day you give notice, so be ready for that day to be your last.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>113</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@craigleveyesq/video/7692193390145899807</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Quiet promotion</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Because the economy isn't doing well, many companies are choosing to quietly promote employees. But what's interesting is that many of these employees are rejecting these promotions.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Because the economy isn't doing well, many companies are choosing to quietly promote employees. But what's interesting is that many of these employees are rejecting these promotions. I'm Evan Lange, with one of Texas's top-rated employment law firms. A quiet promotion means more work, more responsibility, maybe a new title, but no raise. It's pitched as a career move, but without the pay, it's mostly extra stress. And watch your classification: if the company suddenly calls you exempt from overtime, make sure your pay and duties actually meet the legal test. Before you say yes, get the new duties and pay in writing. If the numbers don't change, ask yourself whether it's really worth it.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>115</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@craigleveyesq/video/7691782516734217503</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Exit interview</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Should an employee attend an exit interview after they've told their company that they are leaving? Or is it really only the company that's gonna benefit?</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Should an employee attend an exit interview after they've told their company that they are leaving? Or is it really only the company that's gonna benefit? I'm Evan Lange, with one of Texas's top-rated employment law firms. In most cases, the company gets far more out of it than you do. You're already leaving, and they want information about your job, your team, your manager, and anything that could become a problem later. You can often politely decline. If you do go, keep it short, professional and positive. Don't vent, don't name names, and don't sign anything, especially a release, until you've had time to review it.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>107</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@craigleveyesq/video/7691416065242549535</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Confidential survey</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>When an employee receives a confidential survey from their company, will their answers remain anonymous or will they get passed on?</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>When an employee receives a confidential survey from their company, will their answers remain anonymous or will they get passed on? I'm Evan Lange, with one of Texas's top-rated employment law firms. Assume your answers can be traced back to you. Even without your name, details like your department, your role or a specific incident can point right to you, especially on a small team. And those answers often land on the desk of the managers you're writing about. If you have a serious issue, like harassment, discrimination or unpaid wages, don't bury it in a survey. Report it to HR in writing. That creates a record, and retaliating against you for it is illegal.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>115</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@craigleveyesq/video/7691045923929066783</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>3 illegal things bosses do</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Here are three illegal things bosses do that sound completely normal, and the third one may surprise you the most.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Here are three illegal things bosses do that sound completely normal, and the third one may surprise you the most. I'm Evan Lange, with one of Texas's top-rated employment law firms. One: retaliation. If you report harassment, discrimination, unpaid wages or a safety issue, they can't punish you with a firing, demotion, cut hours or sudden bad reviews. Two: unpaid time. If you're hourly, work before your shift or through an auto-deducted lunch generally has to be paid. Three, and HR hopes you never learn this one: for most private-sector employees, federal law protects your right to discuss your pay with coworkers. Save the policies, track your hours, and write down dates.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>112</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@top.law.assist/video/7690709376595774733</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>3 ways companies fire</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>When a company decides to fire an employee and they know they might get sued by that person, they take three approaches to termination.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>When a company decides to fire an employee and they know they might get sued by that person, they take three approaches to termination. I'm Evan Lange, with one of Texas's top-rated employment law firms. First, the quick firing: no warning, no paper trail. They just do it and hope you don't sue. Second, the numbers game: they fold you into a layoff or reduction in force so a targeted firing looks like a business decision. Third, the slow push: micromanaging, write-ups and bad reviews, sometimes for months, hoping you'll quit. If you don't, they fire you. If this is happening, especially after you complained or took leave, start documenting everything now.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>112</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@craigleveyesq/video/7690672205608307998</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>They want you to resign</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>If your employer does one of the following things to you, they probably want you to resign. And if you don't resign, they will likely fire you.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>If your employer does one of the following things to you, they probably want you to resign. And if you don't resign, they will likely fire you. I'm Evan Lange, with one of Texas's top-rated employment law firms. A sudden bad review, written warnings or a PIP. Your hours or pay get cut, your bonus disappears, you're left out of meetings, or decisions that used to be yours get taken away. Or your manager starts asking, are you sure you're happy here? These moves are designed to make you leave on your own. Before you quit, know this: resigning can make it harder to get unemployment benefits in Texas. Document everything and get legal advice first.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>116</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@craigleveyesq/video/7689951303048383774</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>3 things I wouldn't do</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Here are three things I would not do as an employee coming from my perspective as an employment lawyer.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Here are three things I would not do as an employee coming from my perspective as an employment lawyer. I'm Evan Lange, with one of Texas's top-rated employment law firms. One: I wouldn't take HR's word that a severance offer is final. If you have legal claims, a lawyer may be able to negotiate more. Two: I wouldn't trust an offer letter that says I'm exempt from overtime. Misclassification happens more than you'd think, and the Fair Labor Standards Act decides, not your job title. Three: I wouldn't assume HR's investigation was thorough just because they found no merit to my complaint. Keep your own records and get a second opinion.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>111</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@craigleveyesq/video/7689564792595483935</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>FMLA</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>When an employee takes FMLA leave from work, they need to understand their rights, because in some cases employers will play games.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>When an employee takes FMLA leave from work, they need to understand their rights, because in some cases employers will play games. I'm Evan Lange, with one of Texas's top-rated employment law firms. FMLA can give eligible employees up to 12 weeks of unpaid, job-protected leave for a serious health condition, a new child, or caring for a family member. When you come back, you're entitled to the same or an equivalent job. What's illegal is interfering with your leave or punishing you for taking it, like a sudden demotion, cut hours or a firing. If you qualify and need the leave, take it, and keep copies of your paperwork and every email about it.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>115</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@craigleveyesq/video/7689194087597051167</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Cost of a layoff</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>So what are the real life costs when somebody is laid off from their job?</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>So what are the real life costs when somebody is laid off from their job? I'm Evan Lange, with one of Texas's top-rated employment law firms. First, the obvious ones: your paycheck, health insurance, retirement contributions and paid time off can disappear overnight. That ripples into missed mortgage payments, lost cars, even moving in with family. Then there are the hidden costs: anxiety, depression, and losing your sense of self-worth, especially when the search drags on. If you've been laid off, review any severance before signing and apply for unemployment with the Texas Workforce Commission right away. And if someone you know is going through it, be patient with them.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>110</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@craigleveyesq/video/7688811622264999199</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>3 things you never want</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>From an employee's perspective, there are three things you never want to have happen at your job.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>From an employee's perspective, there are three things you never want to have happen at your job. I'm Evan Lange, with one of Texas's top-rated employment law firms. One: getting a PIP. It often means the company is already planning your exit. Two: getting moved from a manager who supports you to one who doesn't. Your manager shapes how leadership sees you, and a hostile one can quietly build a case against you. Three: being asked to train a new hire on all your duties when nobody has mentioned a promotion or transfer. You might be training your replacement. If any of these happen, start keeping notes and save your reviews.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>111</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@craigleveyesq/video/7686617058754301214</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Illegal termination signs</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>3 warning signs your termination was actually illegal.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>3 warning signs your termination was actually illegal. I'm Evan Lange, with one of Texas's top-rated employment law firms. One: you were fired right after you complained about harassment, discrimination, unpaid wages or a safety issue. That timing can point to retaliation. Two: you were treated worse than coworkers because of your race, sex, age, religion, disability or pregnancy. Federal and Texas law prohibit that. Three: they still owe you money, like unpaid overtime, commissions or a final paycheck. There are strict deadlines to act. If this sounds familiar, you don't need to be sure you have a case. Just talk to an employment lawyer.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>105</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@lawyer.vince/video/7638673445957438733</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>

</xml_diff>

<commit_message>
Update Evan Lange intro line in 45-second scripts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012RwHDQ9KSjMEpyGbxMwsiX
</commit_message>
<xml_diff>
--- a/tiktok_scripts.xlsx
+++ b/tiktok_scripts.xlsx
@@ -492,14 +492,14 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>When an employee receives a PIP, also known as a performance improvement plan, in most cases, they will be fired. I'm Evan Lange, with one of Texas's top-rated employment law firms. A PIP lists the areas where you're supposedly falling short and gives you a deadline, often 30, 60 or 90 days, to fix them. The problem? Many times the decision has already been made, and the PIP becomes the company's proof that they warned you. So if you get one, take it seriously. Keep copies of everything, respond in writing to anything inaccurate, and if it showed up right after you complained or asked for leave, talk to an employment lawyer before your deadline runs out.</t>
+          <t>When an employee receives a PIP, also known as a performance improvement plan, in most cases, they will be fired. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. A PIP lists the areas where you're supposedly falling short and gives you a deadline, often 30, 60 or 90 days, to fix them. The problem? Many times the decision has already been made, and the PIP becomes the company's proof that they warned you. So if you get one, take it seriously. Keep copies of everything, respond in writing to anything inaccurate, and if it showed up right after you complained or asked for leave, talk to an employment lawyer before your deadline runs out.</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -523,14 +523,14 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Can you get fired by your company because you have more than one job? In many cases the answer is yes. I'm Evan Lange, with one of Texas's top-rated employment law firms. Texas is an at-will state, so your employer can let you go for almost any reason that isn't illegal, and having a second job isn't a protected reason. Check your handbook for a moonlighting or outside-employment policy, and read your offer letter for conflict-of-interest or non-compete language. The biggest risks: working for a competitor, using company time or equipment, or letting your performance slip. Not sure? Get approval in writing before you start.</t>
+          <t>Can you get fired by your company because you have more than one job? In many cases the answer is yes. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. Texas is an at-will state, so your employer can let you go for almost any reason that isn't illegal, and having a second job isn't a protected reason. Check your handbook for a moonlighting or outside-employment policy, and read your offer letter for conflict-of-interest or non-compete language. The biggest risks: working for a competitor, using company time or equipment, or letting your performance slip. Not sure? Get approval in writing before you start.</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -554,11 +554,11 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>If I was an employee that was about to resign from their job, here are three things that I would not do. I'm Evan Lange, with one of Texas's top-rated employment law firms. One: don't give notice until your new offer is signed and your background check has cleared. If the new job falls through, you could end up with nothing. Two: don't pick your last day at random. Check when bonuses, commissions and vesting dates hit so you don't leave earned money behind. Three: don't count on working out your two weeks. Many employers can end things the day you give notice, so be ready for that day to be your last.</t>
+          <t>If I was an employee that was about to resign from their job, here are three things that I would not do. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. One: don't give notice until your new offer is signed and your background check has cleared. If the new job falls through, you could end up with nothing. Two: don't pick your last day at random. Check when bonuses, commissions and vesting dates hit so you don't leave earned money behind. Three: don't count on working out your two weeks. Many employers can end things the day you give notice, so be ready for that day to be your last.</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>37</v>
@@ -585,14 +585,14 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Because the economy isn't doing well, many companies are choosing to quietly promote employees. But what's interesting is that many of these employees are rejecting these promotions. I'm Evan Lange, with one of Texas's top-rated employment law firms. A quiet promotion means more work, more responsibility, maybe a new title, but no raise. It's pitched as a career move, but without the pay, it's mostly extra stress. And watch your classification: if the company suddenly calls you exempt from overtime, make sure your pay and duties actually meet the legal test. Before you say yes, get the new duties and pay in writing. If the numbers don't change, ask yourself whether it's really worth it.</t>
+          <t>Because the economy isn't doing well, many companies are choosing to quietly promote employees. But what's interesting is that many of these employees are rejecting these promotions. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. A quiet promotion means more work, more responsibility, maybe a new title, but no raise. It's pitched as a career move, but without the pay, it's mostly extra stress. And watch your classification: if the company suddenly calls you exempt from overtime, make sure your pay and duties actually meet the legal test. Before you say yes, get the new duties and pay in writing. If the numbers don't change, ask yourself whether it's really worth it.</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
@@ -616,14 +616,14 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Should an employee attend an exit interview after they've told their company that they are leaving? Or is it really only the company that's gonna benefit? I'm Evan Lange, with one of Texas's top-rated employment law firms. In most cases, the company gets far more out of it than you do. You're already leaving, and they want information about your job, your team, your manager, and anything that could become a problem later. You can often politely decline. If you do go, keep it short, professional and positive. Don't vent, don't name names, and don't sign anything, especially a release, until you've had time to review it.</t>
+          <t>Should an employee attend an exit interview after they've told their company that they are leaving? Or is it really only the company that's gonna benefit? I'm Evan Lange, and I own one of Texas's top-rated employment law firms. In most cases, the company gets far more out of it than you do. You're already leaving, and they want information about your job, your team, your manager, and anything that could become a problem later. You can often politely decline. If you do go, keep it short, professional and positive. Don't vent, don't name names, and don't sign anything, especially a release, until you've had time to review it.</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -647,14 +647,14 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>When an employee receives a confidential survey from their company, will their answers remain anonymous or will they get passed on? I'm Evan Lange, with one of Texas's top-rated employment law firms. Assume your answers can be traced back to you. Even without your name, details like your department, your role or a specific incident can point right to you, especially on a small team. And those answers often land on the desk of the managers you're writing about. If you have a serious issue, like harassment, discrimination or unpaid wages, don't bury it in a survey. Report it to HR in writing. That creates a record, and retaliating against you for it is illegal.</t>
+          <t>When an employee receives a confidential survey from their company, will their answers remain anonymous or will they get passed on? I'm Evan Lange, and I own one of Texas's top-rated employment law firms. Assume your answers can be traced back to you. Even without your name, details like your department, your role or a specific incident can point right to you, especially on a small team. And those answers often land on the desk of the managers you're writing about. If you have a serious issue, like harassment, discrimination or unpaid wages, don't bury it in a survey. Report it to HR in writing. That creates a record, and retaliating against you for it is illegal.</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
@@ -678,14 +678,14 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Here are three illegal things bosses do that sound completely normal, and the third one may surprise you the most. I'm Evan Lange, with one of Texas's top-rated employment law firms. One: retaliation. If you report harassment, discrimination, unpaid wages or a safety issue, they can't punish you with a firing, demotion, cut hours or sudden bad reviews. Two: unpaid time. If you're hourly, work before your shift or through an auto-deducted lunch generally has to be paid. Three, and HR hopes you never learn this one: for most private-sector employees, federal law protects your right to discuss your pay with coworkers. Save the policies, track your hours, and write down dates.</t>
+          <t>Here are three illegal things bosses do that sound completely normal, and the third one may surprise you the most. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. One: retaliation. If you report harassment, discrimination, unpaid wages or a safety issue, they can't punish you with a firing, demotion, cut hours or sudden bad reviews. Two: unpaid time. If you're hourly, work before your shift or through an auto-deducted lunch generally has to be paid. Three, and HR hopes you never learn this one: for most private-sector employees, federal law protects your right to discuss your pay with coworkers. Save the policies, track your hours, and write down dates.</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -709,14 +709,14 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>When a company decides to fire an employee and they know they might get sued by that person, they take three approaches to termination. I'm Evan Lange, with one of Texas's top-rated employment law firms. First, the quick firing: no warning, no paper trail. They just do it and hope you don't sue. Second, the numbers game: they fold you into a layoff or reduction in force so a targeted firing looks like a business decision. Third, the slow push: micromanaging, write-ups and bad reviews, sometimes for months, hoping you'll quit. If you don't, they fire you. If this is happening, especially after you complained or took leave, start documenting everything now.</t>
+          <t>When a company decides to fire an employee and they know they might get sued by that person, they take three approaches to termination. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. First, the quick firing: no warning, no paper trail. They just do it and hope you don't sue. Second, the numbers game: they fold you into a layoff or reduction in force so a targeted firing looks like a business decision. Third, the slow push: micromanaging, write-ups and bad reviews, sometimes for months, hoping you'll quit. If you don't, they fire you. If this is happening, especially after you complained or took leave, start documenting everything now.</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
@@ -740,11 +740,11 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>If your employer does one of the following things to you, they probably want you to resign. And if you don't resign, they will likely fire you. I'm Evan Lange, with one of Texas's top-rated employment law firms. A sudden bad review, written warnings or a PIP. Your hours or pay get cut, your bonus disappears, you're left out of meetings, or decisions that used to be yours get taken away. Or your manager starts asking, are you sure you're happy here? These moves are designed to make you leave on your own. Before you quit, know this: resigning can make it harder to get unemployment benefits in Texas. Document everything and get legal advice first.</t>
+          <t>If your employer does one of the following things to you, they probably want you to resign. And if you don't resign, they will likely fire you. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. A sudden bad review, written warnings or a PIP. Your hours or pay get cut, your bonus disappears, you're left out of meetings, or decisions that used to be yours get taken away. Or your manager starts asking, are you sure you're happy here? These moves are designed to make you leave on your own. Before you quit, know this: resigning can make it harder to get unemployment benefits in Texas. Document everything and get legal advice first.</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>38</v>
@@ -771,14 +771,14 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Here are three things I would not do as an employee coming from my perspective as an employment lawyer. I'm Evan Lange, with one of Texas's top-rated employment law firms. One: I wouldn't take HR's word that a severance offer is final. If you have legal claims, a lawyer may be able to negotiate more. Two: I wouldn't trust an offer letter that says I'm exempt from overtime. Misclassification happens more than you'd think, and the Fair Labor Standards Act decides, not your job title. Three: I wouldn't assume HR's investigation was thorough just because they found no merit to my complaint. Keep your own records and get a second opinion.</t>
+          <t>Here are three things I would not do as an employee coming from my perspective as an employment lawyer. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. One: I wouldn't take HR's word that a severance offer is final. If you have legal claims, a lawyer may be able to negotiate more. Two: I wouldn't trust an offer letter that says I'm exempt from overtime. Misclassification happens more than you'd think, and the Fair Labor Standards Act decides, not your job title. Three: I wouldn't assume HR's investigation was thorough just because they found no merit to my complaint. Keep your own records and get a second opinion.</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
@@ -802,14 +802,14 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>When an employee takes FMLA leave from work, they need to understand their rights, because in some cases employers will play games. I'm Evan Lange, with one of Texas's top-rated employment law firms. FMLA can give eligible employees up to 12 weeks of unpaid, job-protected leave for a serious health condition, a new child, or caring for a family member. When you come back, you're entitled to the same or an equivalent job. What's illegal is interfering with your leave or punishing you for taking it, like a sudden demotion, cut hours or a firing. If you qualify and need the leave, take it, and keep copies of your paperwork and every email about it.</t>
+          <t>When an employee takes FMLA leave from work, they need to understand their rights, because in some cases employers will play games. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. FMLA can give eligible employees up to 12 weeks of unpaid, job-protected leave for a serious health condition, a new child, or caring for a family member. When you come back, you're entitled to the same or an equivalent job. What's illegal is interfering with your leave or punishing you for taking it, like a sudden demotion, cut hours or a firing. If you qualify and need the leave, take it, and keep copies of your paperwork and every email about it.</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
@@ -833,11 +833,11 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>So what are the real life costs when somebody is laid off from their job? I'm Evan Lange, with one of Texas's top-rated employment law firms. First, the obvious ones: your paycheck, health insurance, retirement contributions and paid time off can disappear overnight. That ripples into missed mortgage payments, lost cars, even moving in with family. Then there are the hidden costs: anxiety, depression, and losing your sense of self-worth, especially when the search drags on. If you've been laid off, review any severance before signing and apply for unemployment with the Texas Workforce Commission right away. And if someone you know is going through it, be patient with them.</t>
+          <t>So what are the real life costs when somebody is laid off from their job? I'm Evan Lange, and I own one of Texas's top-rated employment law firms. First, the obvious ones: your paycheck, health insurance, retirement contributions and paid time off can disappear overnight. That ripples into missed mortgage payments, lost cars, even moving in with family. Then there are the hidden costs: anxiety, depression, and losing your sense of self-worth, especially when the search drags on. If you've been laid off, review any severance before signing and apply for unemployment with the Texas Workforce Commission right away. And if someone you know is going through it, be patient with them.</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F13" s="2" t="n">
         <v>36</v>
@@ -864,14 +864,14 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>From an employee's perspective, there are three things you never want to have happen at your job. I'm Evan Lange, with one of Texas's top-rated employment law firms. One: getting a PIP. It often means the company is already planning your exit. Two: getting moved from a manager who supports you to one who doesn't. Your manager shapes how leadership sees you, and a hostile one can quietly build a case against you. Three: being asked to train a new hire on all your duties when nobody has mentioned a promotion or transfer. You might be training your replacement. If any of these happen, start keeping notes and save your reviews.</t>
+          <t>From an employee's perspective, there are three things you never want to have happen at your job. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. One: getting a PIP. It often means the company is already planning your exit. Two: getting moved from a manager who supports you to one who doesn't. Your manager shapes how leadership sees you, and a hostile one can quietly build a case against you. Three: being asked to train a new hire on all your duties when nobody has mentioned a promotion or transfer. You might be training your replacement. If any of these happen, start keeping notes and save your reviews.</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
@@ -895,14 +895,14 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>3 warning signs your termination was actually illegal. I'm Evan Lange, with one of Texas's top-rated employment law firms. One: you were fired right after you complained about harassment, discrimination, unpaid wages or a safety issue. That timing can point to retaliation. Two: you were treated worse than coworkers because of your race, sex, age, religion, disability or pregnancy. Federal and Texas law prohibit that. Three: they still owe you money, like unpaid overtime, commissions or a final paycheck. There are strict deadlines to act. If this sounds familiar, you don't need to be sure you have a case. Just talk to an employment lawyer.</t>
+          <t>3 warning signs your termination was actually illegal. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. One: you were fired right after you complained about harassment, discrimination, unpaid wages or a safety issue. That timing can point to retaliation. Two: you were treated worse than coworkers because of your race, sex, age, religion, disability or pregnancy. Federal and Texas law prohibit that. Three: they still owe you money, like unpaid overtime, commissions or a final paycheck. There are strict deadlines to act. If this sounds familiar, you don't need to be sure you have a case. Just talk to an employment lawyer.</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Replace hook column with post captions in 45-second scripts sheet
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012RwHDQ9KSjMEpyGbxMwsiX
</commit_message>
<xml_diff>
--- a/tiktok_scripts.xlsx
+++ b/tiktok_scripts.xlsx
@@ -432,7 +432,7 @@
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
     <col width="100" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -452,7 +452,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Hook (sin cambios)</t>
+          <t>Caption (para publicar)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -487,7 +487,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>When an employee receives a PIP, also known as a performance improvement plan, in most cases, they will be fired.</t>
+          <t>Got a PIP? It might not be the fresh start your employer says it is. Here's what to do before the deadline hits. 📄 #employmentlaw #texaslawyer #workplacerights #employeerights #evanlange #pip</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -518,7 +518,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Can you get fired by your company because you have more than one job? In many cases the answer is yes.</t>
+          <t>Side hustle + full-time job = risk? In Texas, it depends on your employer's policies. Check these before you start. 💼 #employmentlaw #texaslawyer #workplacerights #employeerights #evanlange #sidehustle</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -549,7 +549,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>If I was an employee that was about to resign from their job, here are three things that I would not do.</t>
+          <t>Thinking about quitting? Don't give notice until you've checked these 3 things. ✋ #employmentlaw #texaslawyer #workplacerights #employeerights #evanlange #resignation</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -580,7 +580,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Because the economy isn't doing well, many companies are choosing to quietly promote employees. But what's interesting is that many of these employees are rejecting these promotions.</t>
+          <t>More work. New title. Same paycheck. Before you accept a 'quiet promotion,' watch this. 👀 #employmentlaw #texaslawyer #workplacerights #employeerights #evanlange #quietpromotion</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -611,7 +611,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Should an employee attend an exit interview after they've told their company that they are leaving? Or is it really only the company that's gonna benefit?</t>
+          <t>Leaving your job? Think twice before you say too much in the exit interview. 🚪 #employmentlaw #texaslawyer #workplacerights #employeerights #evanlange #exitinterview</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -642,7 +642,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>When an employee receives a confidential survey from their company, will their answers remain anonymous or will they get passed on?</t>
+          <t>That 'anonymous' employee survey might not be as anonymous as you think. 🤫 #employmentlaw #texaslawyer #workplacerights #employeerights #evanlange #hr</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -673,7 +673,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Here are three illegal things bosses do that sound completely normal, and the third one may surprise you the most.</t>
+          <t>These happen at normal-looking companies every day, and they're illegal. Number 3 surprises most people. ⚖️ #employmentlaw #texaslawyer #workplacerights #employeerights #evanlange #knowyourrights</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>When a company decides to fire an employee and they know they might get sued by that person, they take three approaches to termination.</t>
+          <t>How companies fire employees they think might sue them. Do you recognize any of these? 🚩 #employmentlaw #texaslawyer #workplacerights #employeerights #evanlange #wrongfultermination</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>If your employer does one of the following things to you, they probably want you to resign. And if you don't resign, they will likely fire you.</t>
+          <t>Your employer may be pushing you out without saying it. Know the signs before you resign. 🚩 #employmentlaw #texaslawyer #workplacerights #employeerights #evanlange #toxicworkplace</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Here are three things I would not do as an employee coming from my perspective as an employment lawyer.</t>
+          <t>Severance, overtime and HR investigations: 3 things I'd never take at face value. 🧐 #employmentlaw #texaslawyer #workplacerights #employeerights #evanlange #severance</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -797,7 +797,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>When an employee takes FMLA leave from work, they need to understand their rights, because in some cases employers will play games.</t>
+          <t>Taking FMLA leave? Know your rights before you go, and when you come back. 🏥 #employmentlaw #texaslawyer #workplacerights #employeerights #evanlange #fmla</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -828,7 +828,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>So what are the real life costs when somebody is laid off from their job?</t>
+          <t>Being laid off costs a lot more than a paycheck. Here's what to do next in Texas. 💔 #employmentlaw #texaslawyer #workplacerights #employeerights #evanlange #layoffs</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>From an employee's perspective, there are three things you never want to have happen at your job.</t>
+          <t>3 things no employee ever wants to hear at work. Has one happened to you? 😬 #employmentlaw #texaslawyer #workplacerights #employeerights #evanlange #worklife</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -890,7 +890,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>3 warning signs your termination was actually illegal.</t>
+          <t>Was your firing actually illegal? Watch for these 3 warning signs. ⚠️ #employmentlaw #texaslawyer #workplacerights #employeerights #evanlange #wrongfultermination</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add closing CTA to 45-second scripts
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012RwHDQ9KSjMEpyGbxMwsiX
</commit_message>
<xml_diff>
--- a/tiktok_scripts.xlsx
+++ b/tiktok_scripts.xlsx
@@ -492,14 +492,14 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>When an employee receives a PIP, also known as a performance improvement plan, in most cases, they will be fired. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. A PIP lists the areas where you're supposedly falling short and gives you a deadline, often 30, 60 or 90 days, to fix them. The problem? Many times the decision has already been made, and the PIP becomes the company's proof that they warned you. So if you get one, take it seriously. Keep copies of everything, respond in writing to anything inaccurate, and if it showed up right after you complained or asked for leave, talk to an employment lawyer before your deadline runs out.</t>
+          <t>When an employee receives a PIP, also known as a performance improvement plan, in most cases, they will be fired. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. A PIP lists the areas where you're supposedly falling short and gives you a deadline, often 30, 60 or 90 days, to fix them. The problem? Many times the decision has already been made, and the PIP becomes the company's proof that they warned you. So if you get one, take it seriously. Keep copies of everything, respond in writing to anything inaccurate, and if it showed up right after you complained or asked for leave, talk to an employment lawyer before your deadline runs out. Follow us for more helpful tips.</t>
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
@@ -523,14 +523,14 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Can you get fired by your company because you have more than one job? In many cases the answer is yes. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. Texas is an at-will state, so your employer can let you go for almost any reason that isn't illegal, and having a second job isn't a protected reason. Check your handbook for a moonlighting or outside-employment policy, and read your offer letter for conflict-of-interest or non-compete language. The biggest risks: working for a competitor, using company time or equipment, or letting your performance slip. Not sure? Get approval in writing before you start.</t>
+          <t>Can you get fired by your company because you have more than one job? In many cases the answer is yes. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. Texas is an at-will state, so your employer can let you go for almost any reason that isn't illegal, and having a second job isn't a protected reason. Check your handbook for a moonlighting or outside-employment policy, and read your offer letter for conflict-of-interest or non-compete language. The biggest risks: working for a competitor, using company time or equipment, or letting your performance slip. Not sure? Get approval in writing before you start. Follow us for more helpful tips.</t>
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
@@ -554,14 +554,14 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>If I was an employee that was about to resign from their job, here are three things that I would not do. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. One: don't give notice until your new offer is signed and your background check has cleared. If the new job falls through, you could end up with nothing. Two: don't pick your last day at random. Check when bonuses, commissions and vesting dates hit so you don't leave earned money behind. Three: don't count on working out your two weeks. Many employers can end things the day you give notice, so be ready for that day to be your last.</t>
+          <t>If I was an employee that was about to resign from their job, here are three things that I would not do. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. One: don't give notice until your new offer is signed and your background check has cleared. If the new job falls through, you could end up with nothing. Two: don't pick your last day at random. Check when bonuses, commissions and vesting dates hit so you don't leave earned money behind. Three: don't count on working out your two weeks. Many employers can end things the day you give notice, so be ready for that day to be your last. Follow us for more helpful tips.</t>
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
@@ -585,14 +585,14 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Because the economy isn't doing well, many companies are choosing to quietly promote employees. But what's interesting is that many of these employees are rejecting these promotions. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. A quiet promotion means more work, more responsibility, maybe a new title, but no raise. It's pitched as a career move, but without the pay, it's mostly extra stress. And watch your classification: if the company suddenly calls you exempt from overtime, make sure your pay and duties actually meet the legal test. Before you say yes, get the new duties and pay in writing. If the numbers don't change, ask yourself whether it's really worth it.</t>
+          <t>Because the economy isn't doing well, many companies are choosing to quietly promote employees. But what's interesting is that many of these employees are rejecting these promotions. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. A quiet promotion means more work, more responsibility, maybe a new title, but no raise. It's pitched as a career move, but without the pay, it's mostly extra stress. And watch your classification: if the company suddenly calls you exempt from overtime, make sure your pay and duties actually meet the legal test. Before you say yes, get the new duties and pay in writing. If the numbers don't change, ask yourself whether it's really worth it. Follow us for more helpful tips.</t>
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
@@ -616,14 +616,14 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Should an employee attend an exit interview after they've told their company that they are leaving? Or is it really only the company that's gonna benefit? I'm Evan Lange, and I own one of Texas's top-rated employment law firms. In most cases, the company gets far more out of it than you do. You're already leaving, and they want information about your job, your team, your manager, and anything that could become a problem later. You can often politely decline. If you do go, keep it short, professional and positive. Don't vent, don't name names, and don't sign anything, especially a release, until you've had time to review it.</t>
+          <t>Should an employee attend an exit interview after they've told their company that they are leaving? Or is it really only the company that's gonna benefit? I'm Evan Lange, and I own one of Texas's top-rated employment law firms. In most cases, the company gets far more out of it than you do. You're already leaving, and they want information about your job, your team, your manager, and anything that could become a problem later. You can often politely decline. If you do go, keep it short, professional and positive. Don't vent, don't name names, and don't sign anything, especially a release, until you've had time to review it. Follow us for more helpful tips.</t>
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
@@ -647,14 +647,14 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>When an employee receives a confidential survey from their company, will their answers remain anonymous or will they get passed on? I'm Evan Lange, and I own one of Texas's top-rated employment law firms. Assume your answers can be traced back to you. Even without your name, details like your department, your role or a specific incident can point right to you, especially on a small team. And those answers often land on the desk of the managers you're writing about. If you have a serious issue, like harassment, discrimination or unpaid wages, don't bury it in a survey. Report it to HR in writing. That creates a record, and retaliating against you for it is illegal.</t>
+          <t>When an employee receives a confidential survey from their company, will their answers remain anonymous or will they get passed on? I'm Evan Lange, and I own one of Texas's top-rated employment law firms. Assume your answers can be traced back to you. Even without your name, details like your department, your role or a specific incident can point right to you, especially on a small team. And those answers often land on the desk of the managers you're writing about. If you have a serious issue, like harassment, discrimination or unpaid wages, don't bury it in a survey. Report it to HR in writing. That creates a record, and retaliating against you for it is illegal. Follow us for more helpful tips.</t>
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
@@ -678,14 +678,14 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Here are three illegal things bosses do that sound completely normal, and the third one may surprise you the most. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. One: retaliation. If you report harassment, discrimination, unpaid wages or a safety issue, they can't punish you with a firing, demotion, cut hours or sudden bad reviews. Two: unpaid time. If you're hourly, work before your shift or through an auto-deducted lunch generally has to be paid. Three, and HR hopes you never learn this one: for most private-sector employees, federal law protects your right to discuss your pay with coworkers. Save the policies, track your hours, and write down dates.</t>
+          <t>Here are three illegal things bosses do that sound completely normal, and the third one may surprise you the most. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. One: retaliation. If you report harassment, discrimination, unpaid wages or a safety issue, they can't punish you with a firing, demotion, cut hours or sudden bad reviews. Two: unpaid time. If you're hourly, work before your shift or through an auto-deducted lunch generally has to be paid. Three, and HR hopes you never learn this one: for most private-sector employees, federal law protects your right to discuss your pay with coworkers. Save the policies, track your hours, and write down dates. Follow us for more helpful tips.</t>
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
@@ -709,14 +709,14 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>When a company decides to fire an employee and they know they might get sued by that person, they take three approaches to termination. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. First, the quick firing: no warning, no paper trail. They just do it and hope you don't sue. Second, the numbers game: they fold you into a layoff or reduction in force so a targeted firing looks like a business decision. Third, the slow push: micromanaging, write-ups and bad reviews, sometimes for months, hoping you'll quit. If you don't, they fire you. If this is happening, especially after you complained or took leave, start documenting everything now.</t>
+          <t>When a company decides to fire an employee and they know they might get sued by that person, they take three approaches to termination. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. First, the quick firing: no warning, no paper trail. They just do it and hope you don't sue. Second, the numbers game: they fold you into a layoff or reduction in force so a targeted firing looks like a business decision. Third, the slow push: micromanaging, write-ups and bad reviews, sometimes for months, hoping you'll quit. If you don't, they fire you. If this is happening, especially after you complained or took leave, start documenting everything now. Follow us for more helpful tips.</t>
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
@@ -740,14 +740,14 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>If your employer does one of the following things to you, they probably want you to resign. And if you don't resign, they will likely fire you. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. A sudden bad review, written warnings or a PIP. Your hours or pay get cut, your bonus disappears, you're left out of meetings, or decisions that used to be yours get taken away. Or your manager starts asking, are you sure you're happy here? These moves are designed to make you leave on your own. Before you quit, know this: resigning can make it harder to get unemployment benefits in Texas. Document everything and get legal advice first.</t>
+          <t>If your employer does one of the following things to you, they probably want you to resign. And if you don't resign, they will likely fire you. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. A sudden bad review, written warnings or a PIP. Your hours or pay get cut, your bonus disappears, you're left out of meetings, or decisions that used to be yours get taken away. Or your manager starts asking, are you sure you're happy here? These moves are designed to make you leave on your own. Before you quit, know this: resigning can make it harder to get unemployment benefits in Texas. Document everything and get legal advice first. Follow us for more helpful tips.</t>
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
@@ -771,14 +771,14 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Here are three things I would not do as an employee coming from my perspective as an employment lawyer. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. One: I wouldn't take HR's word that a severance offer is final. If you have legal claims, a lawyer may be able to negotiate more. Two: I wouldn't trust an offer letter that says I'm exempt from overtime. Misclassification happens more than you'd think, and the Fair Labor Standards Act decides, not your job title. Three: I wouldn't assume HR's investigation was thorough just because they found no merit to my complaint. Keep your own records and get a second opinion.</t>
+          <t>Here are three things I would not do as an employee coming from my perspective as an employment lawyer. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. One: I wouldn't take HR's word that a severance offer is final. If you have legal claims, a lawyer may be able to negotiate more. Two: I wouldn't trust an offer letter that says I'm exempt from overtime. Misclassification happens more than you'd think, and the Fair Labor Standards Act decides, not your job title. Three: I wouldn't assume HR's investigation was thorough just because they found no merit to my complaint. Keep your own records and get a second opinion. Follow us for more helpful tips.</t>
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
@@ -802,14 +802,14 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>When an employee takes FMLA leave from work, they need to understand their rights, because in some cases employers will play games. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. FMLA can give eligible employees up to 12 weeks of unpaid, job-protected leave for a serious health condition, a new child, or caring for a family member. When you come back, you're entitled to the same or an equivalent job. What's illegal is interfering with your leave or punishing you for taking it, like a sudden demotion, cut hours or a firing. If you qualify and need the leave, take it, and keep copies of your paperwork and every email about it.</t>
+          <t>When an employee takes FMLA leave from work, they need to understand their rights, because in some cases employers will play games. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. FMLA can give eligible employees up to 12 weeks of unpaid, job-protected leave for a serious health condition, a new child, or caring for a family member. When you come back, you're entitled to the same or an equivalent job. What's illegal is interfering with your leave or punishing you for taking it, like a sudden demotion, cut hours or a firing. If you qualify and need the leave, take it, and keep copies of your paperwork and every email about it. Follow us for more helpful tips.</t>
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
@@ -833,14 +833,14 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>So what are the real life costs when somebody is laid off from their job? I'm Evan Lange, and I own one of Texas's top-rated employment law firms. First, the obvious ones: your paycheck, health insurance, retirement contributions and paid time off can disappear overnight. That ripples into missed mortgage payments, lost cars, even moving in with family. Then there are the hidden costs: anxiety, depression, and losing your sense of self-worth, especially when the search drags on. If you've been laid off, review any severance before signing and apply for unemployment with the Texas Workforce Commission right away. And if someone you know is going through it, be patient with them.</t>
+          <t>So what are the real life costs when somebody is laid off from their job? I'm Evan Lange, and I own one of Texas's top-rated employment law firms. First, the obvious ones: your paycheck, health insurance, retirement contributions and paid time off can disappear overnight. That ripples into missed mortgage payments, lost cars, even moving in with family. Then there are the hidden costs: anxiety, depression, and losing your sense of self-worth, especially when the search drags on. If you've been laid off, review any severance before signing and apply for unemployment with the Texas Workforce Commission right away. And if someone you know is going through it, be patient with them. Follow us for more helpful tips.</t>
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
@@ -864,14 +864,14 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>From an employee's perspective, there are three things you never want to have happen at your job. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. One: getting a PIP. It often means the company is already planning your exit. Two: getting moved from a manager who supports you to one who doesn't. Your manager shapes how leadership sees you, and a hostile one can quietly build a case against you. Three: being asked to train a new hire on all your duties when nobody has mentioned a promotion or transfer. You might be training your replacement. If any of these happen, start keeping notes and save your reviews.</t>
+          <t>From an employee's perspective, there are three things you never want to have happen at your job. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. One: getting a PIP. It often means the company is already planning your exit. Two: getting moved from a manager who supports you to one who doesn't. Your manager shapes how leadership sees you, and a hostile one can quietly build a case against you. Three: being asked to train a new hire on all your duties when nobody has mentioned a promotion or transfer. You might be training your replacement. If any of these happen, start keeping notes and save your reviews. Follow us for more helpful tips.</t>
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
@@ -895,14 +895,14 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>3 warning signs your termination was actually illegal. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. One: you were fired right after you complained about harassment, discrimination, unpaid wages or a safety issue. That timing can point to retaliation. Two: you were treated worse than coworkers because of your race, sex, age, religion, disability or pregnancy. Federal and Texas law prohibit that. Three: they still owe you money, like unpaid overtime, commissions or a final paycheck. There are strict deadlines to act. If this sounds familiar, you don't need to be sure you have a case. Just talk to an employment lawyer.</t>
+          <t>3 warning signs your termination was actually illegal. I'm Evan Lange, and I own one of Texas's top-rated employment law firms. One: you were fired right after you complained about harassment, discrimination, unpaid wages or a safety issue. That timing can point to retaliation. Two: you were treated worse than coworkers because of your race, sex, age, religion, disability or pregnancy. Federal and Texas law prohibit that. Three: they still owe you money, like unpaid overtime, commissions or a final paycheck. There are strict deadlines to act. If this sounds familiar, you don't need to be sure you have a case. Just talk to an employment lawyer. Follow us for more helpful tips.</t>
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>

</xml_diff>